<commit_message>
SCRUM-32: Remove PII from tests and docs; tolerate BOM in sample product files
- Tests no longer embed member names or postal codes; the duplicate-member test reads the row from the file at runtime
- Member 360 PRD and data dictionary show "(PII - not shown)" as examples for first_name, last_name, postal_code
- Sample product header checks read with utf-8-sig so a byte-order mark doesn't break them
- Unit test case documents regenerated (130/130, 127/127); tasks 8.2 and 8.3 ticked; tools/.gitignore added

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/DP_Fraud_Case/Unit_Test_Cases_Fraud_Case.xlsx
+++ b/output/DP_Fraud_Case/Unit_Test_Cases_Fraud_Case.xlsx
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="3">
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.21</v>
+        <v>0.225</v>
       </c>
     </row>
     <row r="6">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08699999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -727,7 +727,7 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="8">
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="10">
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="H10" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="11">
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0.188</v>
+        <v>0.197</v>
       </c>
     </row>
     <row r="13">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="H13" s="2" t="n">
-        <v>0.161</v>
+        <v>0.212</v>
       </c>
     </row>
     <row r="14">
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="H14" s="2" t="n">
-        <v>0.176</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="15">
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>0.183</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="16">
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="25">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>test_parse_value_by_type[CHAR(5)-28202-28202]</t>
+          <t>test_parse_value_by_type[CHAR(5)-12345-12345]</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Parse value by type [CHAR(5)-28202-28202]</t>
+          <t>Parse value by type [CHAR(5)-12345-12345]</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="41">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="H41" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="42">
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="H42" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="43">
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="44">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H44" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="45">
@@ -2247,7 +2247,7 @@
         </is>
       </c>
       <c r="H45" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="46">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="H46" s="2" t="n">
-        <v>0.178</v>
+        <v>0.192</v>
       </c>
     </row>
     <row r="47">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="H47" s="2" t="n">
-        <v>0.205</v>
+        <v>0.183</v>
       </c>
     </row>
     <row r="48">
@@ -2367,7 +2367,7 @@
         </is>
       </c>
       <c r="H48" s="2" t="n">
-        <v>0.193</v>
+        <v>0.181</v>
       </c>
     </row>
     <row r="49">
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="H49" s="2" t="n">
-        <v>0.203</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="50">
@@ -2447,7 +2447,7 @@
         </is>
       </c>
       <c r="H50" s="2" t="n">
-        <v>0.19</v>
+        <v>0.186</v>
       </c>
     </row>
     <row r="51">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="H51" s="2" t="n">
-        <v>0.184</v>
+        <v>0.181</v>
       </c>
     </row>
     <row r="52">
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="H52" s="2" t="n">
-        <v>0.188</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="53">
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>0.184</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="54">
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="H54" s="2" t="n">
-        <v>0.109</v>
+        <v>0.108</v>
       </c>
     </row>
     <row r="55">
@@ -2687,7 +2687,7 @@
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="57">
@@ -2727,7 +2727,7 @@
         </is>
       </c>
       <c r="H57" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="58">
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="H59" s="2" t="n">
-        <v>0.384</v>
+        <v>0.199</v>
       </c>
     </row>
     <row r="60">
@@ -2847,7 +2847,7 @@
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="61">
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="H68" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="69">
@@ -3207,7 +3207,7 @@
         </is>
       </c>
       <c r="H69" s="2" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="70">
@@ -3327,7 +3327,7 @@
         </is>
       </c>
       <c r="H72" s="2" t="n">
-        <v>0.133</v>
+        <v>0.115</v>
       </c>
     </row>
     <row r="73">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="H74" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="75">
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="H75" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="76">
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="H76" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="77">
@@ -3527,7 +3527,7 @@
         </is>
       </c>
       <c r="H77" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="78">
@@ -3687,7 +3687,7 @@
         </is>
       </c>
       <c r="H81" s="2" t="n">
-        <v>0.027</v>
+        <v>0.057</v>
       </c>
     </row>
     <row r="82">
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="H82" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="83">
@@ -3767,7 +3767,7 @@
         </is>
       </c>
       <c r="H83" s="2" t="n">
-        <v>0.005</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="84">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H84" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="85">
@@ -3847,7 +3847,7 @@
         </is>
       </c>
       <c r="H85" s="2" t="n">
-        <v>0.005</v>
+        <v>0.032</v>
       </c>
     </row>
     <row r="86">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="H86" s="2" t="n">
-        <v>0.232</v>
+        <v>0.199</v>
       </c>
     </row>
     <row r="87">
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="H87" s="2" t="n">
-        <v>0.235</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="88">
@@ -4047,7 +4047,7 @@
         </is>
       </c>
       <c r="H90" s="2" t="n">
-        <v>0.111</v>
+        <v>0.108</v>
       </c>
     </row>
     <row r="91">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="H91" s="2" t="n">
-        <v>0.106</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="92">
@@ -4127,7 +4127,7 @@
         </is>
       </c>
       <c r="H92" s="2" t="n">
-        <v>0.232</v>
+        <v>0.471</v>
       </c>
     </row>
     <row r="93">
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="H93" s="2" t="n">
-        <v>0.222</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="94">
@@ -4247,7 +4247,7 @@
         </is>
       </c>
       <c r="H95" s="2" t="n">
-        <v>0.209</v>
+        <v>0.182</v>
       </c>
     </row>
     <row r="96">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="H96" s="2" t="n">
-        <v>0.163</v>
+        <v>0.139</v>
       </c>
     </row>
     <row r="97">
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="H97" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="98">
@@ -4367,7 +4367,7 @@
         </is>
       </c>
       <c r="H98" s="2" t="n">
-        <v>0.136</v>
+        <v>0.115</v>
       </c>
     </row>
     <row r="99">
@@ -4407,7 +4407,7 @@
         </is>
       </c>
       <c r="H99" s="2" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="100">
@@ -5007,7 +5007,7 @@
         </is>
       </c>
       <c r="H114" s="2" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="115">
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="H119" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="120">
@@ -5447,7 +5447,7 @@
         </is>
       </c>
       <c r="H125" s="2" t="n">
-        <v>0.034</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="126">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="H126" s="2" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="127">
@@ -5527,7 +5527,7 @@
         </is>
       </c>
       <c r="H127" s="2" t="n">
-        <v>0.023</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="128">
@@ -5567,7 +5567,7 @@
         </is>
       </c>
       <c r="H128" s="2" t="n">
-        <v>0.011</v>
+        <v>0.007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>